<commit_message>
PFA-C, DCF1-11, UI, BUG FIXES
</commit_message>
<xml_diff>
--- a/assets/downloadables/DCF_Form_4.xlsx
+++ b/assets/downloadables/DCF_Form_4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\Systems\dti_web_app_v2\assets\downloadables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88CC9170-D0C1-4E76-981F-79738414C02C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F893D271-E2ED-414F-9C02-7FC6DE48EFB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="form4" sheetId="1" r:id="rId1"/>
@@ -111,22 +111,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">ACTIVITY DURATION
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(Day, Month, Year)</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Name of Resource Person/Facilitator/BDSP
 </t>
     </r>
@@ -565,6 +549,22 @@
   </si>
   <si>
     <t>enter firstname middle name last name if multiple data add comma (ex. Fullname1, Fullname2, Fullname3)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ACTIVITY DURATION
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(YYYY-MM-DD)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -835,25 +835,10 @@
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -866,6 +851,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1186,831 +1186,831 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="30"/>
-      <c r="P2" s="30"/>
-      <c r="Q2" s="30"/>
-      <c r="R2" s="30"/>
-      <c r="S2" s="30"/>
-      <c r="T2" s="30"/>
-      <c r="U2" s="30"/>
-      <c r="V2" s="30"/>
-      <c r="W2" s="30"/>
-      <c r="X2" s="30"/>
-      <c r="Y2" s="30"/>
-      <c r="Z2" s="30"/>
-      <c r="AA2" s="30"/>
-      <c r="AB2" s="30"/>
-      <c r="AC2" s="30"/>
-      <c r="AD2" s="30"/>
-      <c r="AE2" s="30"/>
-      <c r="AF2" s="30"/>
-      <c r="AG2" s="30"/>
-      <c r="AH2" s="30"/>
-      <c r="AI2" s="30"/>
-      <c r="AJ2" s="30"/>
-      <c r="AK2" s="31" t="s">
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
+      <c r="K2" s="40"/>
+      <c r="L2" s="40"/>
+      <c r="M2" s="40"/>
+      <c r="N2" s="40"/>
+      <c r="O2" s="40"/>
+      <c r="P2" s="40"/>
+      <c r="Q2" s="40"/>
+      <c r="R2" s="40"/>
+      <c r="S2" s="40"/>
+      <c r="T2" s="40"/>
+      <c r="U2" s="40"/>
+      <c r="V2" s="40"/>
+      <c r="W2" s="40"/>
+      <c r="X2" s="40"/>
+      <c r="Y2" s="40"/>
+      <c r="Z2" s="40"/>
+      <c r="AA2" s="40"/>
+      <c r="AB2" s="40"/>
+      <c r="AC2" s="40"/>
+      <c r="AD2" s="40"/>
+      <c r="AE2" s="40"/>
+      <c r="AF2" s="40"/>
+      <c r="AG2" s="40"/>
+      <c r="AH2" s="40"/>
+      <c r="AI2" s="40"/>
+      <c r="AJ2" s="40"/>
+      <c r="AK2" s="37" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:37" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C3" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="32" t="s">
+      <c r="D3" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="32" t="s">
+      <c r="E3" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="32" t="s">
+      <c r="F3" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="33" t="s">
+      <c r="G3" s="38" t="s">
+        <v>157</v>
+      </c>
+      <c r="H3" s="39"/>
+      <c r="I3" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="J3" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="K3" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="H3" s="34"/>
-      <c r="I3" s="32" t="s">
+      <c r="L3" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="M3" s="38" t="s">
+        <v>10</v>
+      </c>
+      <c r="N3" s="39"/>
+      <c r="O3" s="38" t="s">
+        <v>12</v>
+      </c>
+      <c r="P3" s="41"/>
+      <c r="Q3" s="39"/>
+      <c r="R3" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="S3" s="41"/>
+      <c r="T3" s="41"/>
+      <c r="U3" s="41"/>
+      <c r="V3" s="39"/>
+      <c r="W3" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="X3" s="41"/>
+      <c r="Y3" s="41"/>
+      <c r="Z3" s="41"/>
+      <c r="AA3" s="41"/>
+      <c r="AB3" s="41"/>
+      <c r="AC3" s="41"/>
+      <c r="AD3" s="41"/>
+      <c r="AE3" s="41"/>
+      <c r="AF3" s="39"/>
+      <c r="AG3" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="AH3" s="41"/>
+      <c r="AI3" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="AJ3" s="40"/>
+      <c r="AK3" s="37"/>
+    </row>
+    <row r="4" spans="1:37" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="M4" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="N4" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="30" t="s">
+        <v>13</v>
+      </c>
+      <c r="P4" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q4" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="R4" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="S4" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="T4" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="U4" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="V4" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="W4" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="X4" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y4" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z4" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA4" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB4" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC4" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD4" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="AE4" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF4" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG4" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="AH4" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="AI4" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="AJ4" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="AK4" s="37"/>
+    </row>
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="A5" s="33">
+        <v>0</v>
+      </c>
+      <c r="B5" s="33">
+        <v>1</v>
+      </c>
+      <c r="C5" s="33">
+        <v>2</v>
+      </c>
+      <c r="D5" s="33">
+        <v>3</v>
+      </c>
+      <c r="E5" s="33">
+        <v>4</v>
+      </c>
+      <c r="F5" s="33">
+        <v>5</v>
+      </c>
+      <c r="G5" s="33">
+        <v>6</v>
+      </c>
+      <c r="H5" s="33">
         <v>7</v>
       </c>
-      <c r="J3" s="32" t="s">
+      <c r="I5" s="33">
         <v>8</v>
       </c>
-      <c r="K3" s="32" t="s">
+      <c r="J5" s="33">
+        <v>9</v>
+      </c>
+      <c r="K5" s="33">
+        <v>10</v>
+      </c>
+      <c r="L5" s="33">
+        <v>11</v>
+      </c>
+      <c r="M5" s="33">
+        <v>12</v>
+      </c>
+      <c r="N5" s="33">
+        <v>13</v>
+      </c>
+      <c r="O5" s="33">
+        <v>14</v>
+      </c>
+      <c r="P5" s="33">
+        <v>15</v>
+      </c>
+      <c r="Q5" s="33">
+        <v>16</v>
+      </c>
+      <c r="R5" s="33">
+        <v>17</v>
+      </c>
+      <c r="S5" s="33">
+        <v>18</v>
+      </c>
+      <c r="T5" s="33">
+        <v>19</v>
+      </c>
+      <c r="U5" s="33">
+        <v>20</v>
+      </c>
+      <c r="V5" s="33">
+        <v>21</v>
+      </c>
+      <c r="W5" s="33">
+        <v>22</v>
+      </c>
+      <c r="X5" s="33">
+        <v>23</v>
+      </c>
+      <c r="Y5" s="33">
+        <v>24</v>
+      </c>
+      <c r="Z5" s="33">
+        <v>25</v>
+      </c>
+      <c r="AA5" s="33">
+        <v>26</v>
+      </c>
+      <c r="AB5" s="33">
+        <v>27</v>
+      </c>
+      <c r="AC5" s="33">
         <v>28</v>
       </c>
-      <c r="L3" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="M3" s="33" t="s">
-        <v>10</v>
-      </c>
-      <c r="N3" s="34"/>
-      <c r="O3" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="P3" s="35"/>
-      <c r="Q3" s="34"/>
-      <c r="R3" s="33" t="s">
-        <v>16</v>
-      </c>
-      <c r="S3" s="35"/>
-      <c r="T3" s="35"/>
-      <c r="U3" s="35"/>
-      <c r="V3" s="34"/>
-      <c r="W3" s="35" t="s">
+      <c r="AD5" s="33">
+        <v>29</v>
+      </c>
+      <c r="AE5" s="33">
+        <v>30</v>
+      </c>
+      <c r="AF5" s="33">
+        <v>31</v>
+      </c>
+      <c r="AG5" s="33">
+        <v>32</v>
+      </c>
+      <c r="AH5" s="33">
+        <v>33</v>
+      </c>
+      <c r="AI5" s="33">
         <v>34</v>
       </c>
-      <c r="X3" s="35"/>
-      <c r="Y3" s="35"/>
-      <c r="Z3" s="35"/>
-      <c r="AA3" s="35"/>
-      <c r="AB3" s="35"/>
-      <c r="AC3" s="35"/>
-      <c r="AD3" s="35"/>
-      <c r="AE3" s="35"/>
-      <c r="AF3" s="34"/>
-      <c r="AG3" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH3" s="35"/>
-      <c r="AI3" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="AJ3" s="30"/>
-      <c r="AK3" s="31"/>
-    </row>
-    <row r="4" spans="1:37" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="32"/>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" s="32" t="s">
-        <v>33</v>
-      </c>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
-      <c r="K4" s="32"/>
-      <c r="L4" s="32" t="s">
-        <v>29</v>
-      </c>
-      <c r="M4" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="N4" s="32" t="s">
-        <v>30</v>
-      </c>
-      <c r="O4" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="P4" s="32" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q4" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="R4" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="S4" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="T4" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="U4" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="V4" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="W4" s="32" t="s">
+      <c r="AJ5" s="33">
         <v>35</v>
       </c>
-      <c r="X4" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="Y4" s="32" t="s">
-        <v>37</v>
-      </c>
-      <c r="Z4" s="36" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA4" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB4" s="36" t="s">
-        <v>42</v>
-      </c>
-      <c r="AC4" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD4" s="36" t="s">
-        <v>43</v>
-      </c>
-      <c r="AE4" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="AF4" s="36" t="s">
-        <v>44</v>
-      </c>
-      <c r="AG4" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="AH4" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="AI4" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="AJ4" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="AK4" s="31"/>
-    </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A5" s="38">
-        <v>0</v>
-      </c>
-      <c r="B5" s="38">
-        <v>1</v>
-      </c>
-      <c r="C5" s="38">
-        <v>2</v>
-      </c>
-      <c r="D5" s="38">
-        <v>3</v>
-      </c>
-      <c r="E5" s="38">
-        <v>4</v>
-      </c>
-      <c r="F5" s="38">
-        <v>5</v>
-      </c>
-      <c r="G5" s="38">
-        <v>6</v>
-      </c>
-      <c r="H5" s="38">
-        <v>7</v>
-      </c>
-      <c r="I5" s="38">
-        <v>8</v>
-      </c>
-      <c r="J5" s="38">
-        <v>9</v>
-      </c>
-      <c r="K5" s="38">
-        <v>10</v>
-      </c>
-      <c r="L5" s="38">
-        <v>11</v>
-      </c>
-      <c r="M5" s="38">
-        <v>12</v>
-      </c>
-      <c r="N5" s="38">
-        <v>13</v>
-      </c>
-      <c r="O5" s="38">
-        <v>14</v>
-      </c>
-      <c r="P5" s="38">
-        <v>15</v>
-      </c>
-      <c r="Q5" s="38">
-        <v>16</v>
-      </c>
-      <c r="R5" s="38">
-        <v>17</v>
-      </c>
-      <c r="S5" s="38">
-        <v>18</v>
-      </c>
-      <c r="T5" s="38">
-        <v>19</v>
-      </c>
-      <c r="U5" s="38">
-        <v>20</v>
-      </c>
-      <c r="V5" s="38">
-        <v>21</v>
-      </c>
-      <c r="W5" s="38">
-        <v>22</v>
-      </c>
-      <c r="X5" s="38">
-        <v>23</v>
-      </c>
-      <c r="Y5" s="38">
-        <v>24</v>
-      </c>
-      <c r="Z5" s="38">
-        <v>25</v>
-      </c>
-      <c r="AA5" s="38">
-        <v>26</v>
-      </c>
-      <c r="AB5" s="38">
-        <v>27</v>
-      </c>
-      <c r="AC5" s="38">
-        <v>28</v>
-      </c>
-      <c r="AD5" s="38">
-        <v>29</v>
-      </c>
-      <c r="AE5" s="38">
-        <v>30</v>
-      </c>
-      <c r="AF5" s="38">
-        <v>31</v>
-      </c>
-      <c r="AG5" s="38">
-        <v>32</v>
-      </c>
-      <c r="AH5" s="38">
-        <v>33</v>
-      </c>
-      <c r="AI5" s="38">
-        <v>34</v>
-      </c>
-      <c r="AJ5" s="38">
-        <v>35</v>
-      </c>
-      <c r="AK5" s="39"/>
+      <c r="AK5" s="34"/>
     </row>
     <row r="6" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A6" s="40"/>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="40"/>
-      <c r="K6" s="40"/>
-      <c r="L6" s="40"/>
-      <c r="M6" s="40"/>
-      <c r="N6" s="40"/>
-      <c r="O6" s="40"/>
-      <c r="P6" s="40"/>
-      <c r="Q6" s="40"/>
-      <c r="R6" s="40"/>
-      <c r="S6" s="40"/>
-      <c r="T6" s="40"/>
-      <c r="U6" s="40"/>
-      <c r="V6" s="40"/>
-      <c r="W6" s="40"/>
-      <c r="X6" s="40"/>
-      <c r="Y6" s="40"/>
-      <c r="Z6" s="40"/>
-      <c r="AA6" s="40"/>
-      <c r="AB6" s="40"/>
-      <c r="AC6" s="40"/>
-      <c r="AD6" s="40"/>
-      <c r="AE6" s="40"/>
-      <c r="AF6" s="40"/>
-      <c r="AG6" s="40"/>
-      <c r="AH6" s="41"/>
-      <c r="AI6" s="40"/>
-      <c r="AJ6" s="40"/>
-      <c r="AK6" s="39"/>
+      <c r="A6" s="35"/>
+      <c r="B6" s="35"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="35"/>
+      <c r="I6" s="35"/>
+      <c r="J6" s="35"/>
+      <c r="K6" s="35"/>
+      <c r="L6" s="35"/>
+      <c r="M6" s="35"/>
+      <c r="N6" s="35"/>
+      <c r="O6" s="35"/>
+      <c r="P6" s="35"/>
+      <c r="Q6" s="35"/>
+      <c r="R6" s="35"/>
+      <c r="S6" s="35"/>
+      <c r="T6" s="35"/>
+      <c r="U6" s="35"/>
+      <c r="V6" s="35"/>
+      <c r="W6" s="35"/>
+      <c r="X6" s="35"/>
+      <c r="Y6" s="35"/>
+      <c r="Z6" s="35"/>
+      <c r="AA6" s="35"/>
+      <c r="AB6" s="35"/>
+      <c r="AC6" s="35"/>
+      <c r="AD6" s="35"/>
+      <c r="AE6" s="35"/>
+      <c r="AF6" s="35"/>
+      <c r="AG6" s="35"/>
+      <c r="AH6" s="36"/>
+      <c r="AI6" s="35"/>
+      <c r="AJ6" s="35"/>
+      <c r="AK6" s="34"/>
     </row>
     <row r="7" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A7" s="40"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="40"/>
-      <c r="H7" s="40"/>
-      <c r="I7" s="40"/>
-      <c r="J7" s="40"/>
-      <c r="K7" s="40"/>
-      <c r="L7" s="40"/>
-      <c r="M7" s="40"/>
-      <c r="N7" s="40"/>
-      <c r="O7" s="40"/>
-      <c r="P7" s="40"/>
-      <c r="Q7" s="40"/>
-      <c r="R7" s="40"/>
-      <c r="S7" s="40"/>
-      <c r="T7" s="40"/>
-      <c r="U7" s="40"/>
-      <c r="V7" s="40"/>
-      <c r="W7" s="40"/>
-      <c r="X7" s="40"/>
-      <c r="Y7" s="40"/>
-      <c r="Z7" s="40"/>
-      <c r="AA7" s="40"/>
-      <c r="AB7" s="40"/>
-      <c r="AC7" s="40"/>
-      <c r="AD7" s="40"/>
-      <c r="AE7" s="40"/>
-      <c r="AF7" s="40"/>
-      <c r="AG7" s="40"/>
-      <c r="AH7" s="41"/>
-      <c r="AI7" s="40"/>
-      <c r="AJ7" s="40"/>
-      <c r="AK7" s="39"/>
+      <c r="A7" s="35"/>
+      <c r="B7" s="35"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
+      <c r="G7" s="35"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="35"/>
+      <c r="J7" s="35"/>
+      <c r="K7" s="35"/>
+      <c r="L7" s="35"/>
+      <c r="M7" s="35"/>
+      <c r="N7" s="35"/>
+      <c r="O7" s="35"/>
+      <c r="P7" s="35"/>
+      <c r="Q7" s="35"/>
+      <c r="R7" s="35"/>
+      <c r="S7" s="35"/>
+      <c r="T7" s="35"/>
+      <c r="U7" s="35"/>
+      <c r="V7" s="35"/>
+      <c r="W7" s="35"/>
+      <c r="X7" s="35"/>
+      <c r="Y7" s="35"/>
+      <c r="Z7" s="35"/>
+      <c r="AA7" s="35"/>
+      <c r="AB7" s="35"/>
+      <c r="AC7" s="35"/>
+      <c r="AD7" s="35"/>
+      <c r="AE7" s="35"/>
+      <c r="AF7" s="35"/>
+      <c r="AG7" s="35"/>
+      <c r="AH7" s="36"/>
+      <c r="AI7" s="35"/>
+      <c r="AJ7" s="35"/>
+      <c r="AK7" s="34"/>
     </row>
     <row r="8" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A8" s="40"/>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
-      <c r="J8" s="40"/>
-      <c r="K8" s="40"/>
-      <c r="L8" s="40"/>
-      <c r="M8" s="40"/>
-      <c r="N8" s="40"/>
-      <c r="O8" s="40"/>
-      <c r="P8" s="40"/>
-      <c r="Q8" s="40"/>
-      <c r="R8" s="40"/>
-      <c r="S8" s="40"/>
-      <c r="T8" s="40"/>
-      <c r="U8" s="40"/>
-      <c r="V8" s="40"/>
-      <c r="W8" s="40"/>
-      <c r="X8" s="40"/>
-      <c r="Y8" s="40"/>
-      <c r="Z8" s="40"/>
-      <c r="AA8" s="40"/>
-      <c r="AB8" s="40"/>
-      <c r="AC8" s="40"/>
-      <c r="AD8" s="40"/>
-      <c r="AE8" s="40"/>
-      <c r="AF8" s="40"/>
-      <c r="AG8" s="40"/>
-      <c r="AH8" s="41"/>
-      <c r="AI8" s="40"/>
-      <c r="AJ8" s="40"/>
-      <c r="AK8" s="39"/>
+      <c r="A8" s="35"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="35"/>
+      <c r="K8" s="35"/>
+      <c r="L8" s="35"/>
+      <c r="M8" s="35"/>
+      <c r="N8" s="35"/>
+      <c r="O8" s="35"/>
+      <c r="P8" s="35"/>
+      <c r="Q8" s="35"/>
+      <c r="R8" s="35"/>
+      <c r="S8" s="35"/>
+      <c r="T8" s="35"/>
+      <c r="U8" s="35"/>
+      <c r="V8" s="35"/>
+      <c r="W8" s="35"/>
+      <c r="X8" s="35"/>
+      <c r="Y8" s="35"/>
+      <c r="Z8" s="35"/>
+      <c r="AA8" s="35"/>
+      <c r="AB8" s="35"/>
+      <c r="AC8" s="35"/>
+      <c r="AD8" s="35"/>
+      <c r="AE8" s="35"/>
+      <c r="AF8" s="35"/>
+      <c r="AG8" s="35"/>
+      <c r="AH8" s="36"/>
+      <c r="AI8" s="35"/>
+      <c r="AJ8" s="35"/>
+      <c r="AK8" s="34"/>
     </row>
     <row r="9" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A9" s="40"/>
-      <c r="B9" s="40"/>
-      <c r="C9" s="40"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="40"/>
-      <c r="F9" s="40"/>
-      <c r="G9" s="40"/>
-      <c r="H9" s="40"/>
-      <c r="I9" s="40"/>
-      <c r="J9" s="40"/>
-      <c r="K9" s="40"/>
-      <c r="L9" s="40"/>
-      <c r="M9" s="40"/>
-      <c r="N9" s="40"/>
-      <c r="O9" s="40"/>
-      <c r="P9" s="40"/>
-      <c r="Q9" s="40"/>
-      <c r="R9" s="40"/>
-      <c r="S9" s="40"/>
-      <c r="T9" s="40"/>
-      <c r="U9" s="40"/>
-      <c r="V9" s="40"/>
-      <c r="W9" s="40"/>
-      <c r="X9" s="40"/>
-      <c r="Y9" s="40"/>
-      <c r="Z9" s="40"/>
-      <c r="AA9" s="40"/>
-      <c r="AB9" s="40"/>
-      <c r="AC9" s="40"/>
-      <c r="AD9" s="40"/>
-      <c r="AE9" s="40"/>
-      <c r="AF9" s="40"/>
-      <c r="AG9" s="40"/>
-      <c r="AH9" s="41"/>
-      <c r="AI9" s="40"/>
-      <c r="AJ9" s="40"/>
-      <c r="AK9" s="39"/>
+      <c r="A9" s="35"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="35"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="35"/>
+      <c r="J9" s="35"/>
+      <c r="K9" s="35"/>
+      <c r="L9" s="35"/>
+      <c r="M9" s="35"/>
+      <c r="N9" s="35"/>
+      <c r="O9" s="35"/>
+      <c r="P9" s="35"/>
+      <c r="Q9" s="35"/>
+      <c r="R9" s="35"/>
+      <c r="S9" s="35"/>
+      <c r="T9" s="35"/>
+      <c r="U9" s="35"/>
+      <c r="V9" s="35"/>
+      <c r="W9" s="35"/>
+      <c r="X9" s="35"/>
+      <c r="Y9" s="35"/>
+      <c r="Z9" s="35"/>
+      <c r="AA9" s="35"/>
+      <c r="AB9" s="35"/>
+      <c r="AC9" s="35"/>
+      <c r="AD9" s="35"/>
+      <c r="AE9" s="35"/>
+      <c r="AF9" s="35"/>
+      <c r="AG9" s="35"/>
+      <c r="AH9" s="36"/>
+      <c r="AI9" s="35"/>
+      <c r="AJ9" s="35"/>
+      <c r="AK9" s="34"/>
     </row>
     <row r="10" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A10" s="40"/>
-      <c r="B10" s="40"/>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="40"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="40"/>
-      <c r="K10" s="40"/>
-      <c r="L10" s="40"/>
-      <c r="M10" s="40"/>
-      <c r="N10" s="40"/>
-      <c r="O10" s="40"/>
-      <c r="P10" s="40"/>
-      <c r="Q10" s="40"/>
-      <c r="R10" s="40"/>
-      <c r="S10" s="40"/>
-      <c r="T10" s="40"/>
-      <c r="U10" s="40"/>
-      <c r="V10" s="40"/>
-      <c r="W10" s="40"/>
-      <c r="X10" s="40"/>
-      <c r="Y10" s="40"/>
-      <c r="Z10" s="40"/>
-      <c r="AA10" s="40"/>
-      <c r="AB10" s="40"/>
-      <c r="AC10" s="40"/>
-      <c r="AD10" s="40"/>
-      <c r="AE10" s="40"/>
-      <c r="AF10" s="40"/>
-      <c r="AG10" s="40"/>
-      <c r="AH10" s="41"/>
-      <c r="AI10" s="40"/>
-      <c r="AJ10" s="40"/>
-      <c r="AK10" s="39"/>
+      <c r="A10" s="35"/>
+      <c r="B10" s="35"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="35"/>
+      <c r="I10" s="35"/>
+      <c r="J10" s="35"/>
+      <c r="K10" s="35"/>
+      <c r="L10" s="35"/>
+      <c r="M10" s="35"/>
+      <c r="N10" s="35"/>
+      <c r="O10" s="35"/>
+      <c r="P10" s="35"/>
+      <c r="Q10" s="35"/>
+      <c r="R10" s="35"/>
+      <c r="S10" s="35"/>
+      <c r="T10" s="35"/>
+      <c r="U10" s="35"/>
+      <c r="V10" s="35"/>
+      <c r="W10" s="35"/>
+      <c r="X10" s="35"/>
+      <c r="Y10" s="35"/>
+      <c r="Z10" s="35"/>
+      <c r="AA10" s="35"/>
+      <c r="AB10" s="35"/>
+      <c r="AC10" s="35"/>
+      <c r="AD10" s="35"/>
+      <c r="AE10" s="35"/>
+      <c r="AF10" s="35"/>
+      <c r="AG10" s="35"/>
+      <c r="AH10" s="36"/>
+      <c r="AI10" s="35"/>
+      <c r="AJ10" s="35"/>
+      <c r="AK10" s="34"/>
     </row>
     <row r="11" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A11" s="40"/>
-      <c r="B11" s="40"/>
-      <c r="C11" s="40"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
-      <c r="H11" s="40"/>
-      <c r="I11" s="40"/>
-      <c r="J11" s="40"/>
-      <c r="K11" s="40"/>
-      <c r="L11" s="40"/>
-      <c r="M11" s="40"/>
-      <c r="N11" s="40"/>
-      <c r="O11" s="40"/>
-      <c r="P11" s="40"/>
-      <c r="Q11" s="40"/>
-      <c r="R11" s="40"/>
-      <c r="S11" s="40"/>
-      <c r="T11" s="40"/>
-      <c r="U11" s="40"/>
-      <c r="V11" s="40"/>
-      <c r="W11" s="40"/>
-      <c r="X11" s="40"/>
-      <c r="Y11" s="40"/>
-      <c r="Z11" s="40"/>
-      <c r="AA11" s="40"/>
-      <c r="AB11" s="40"/>
-      <c r="AC11" s="40"/>
-      <c r="AD11" s="40"/>
-      <c r="AE11" s="40"/>
-      <c r="AF11" s="40"/>
-      <c r="AG11" s="40"/>
-      <c r="AH11" s="41"/>
-      <c r="AI11" s="40"/>
-      <c r="AJ11" s="40"/>
-      <c r="AK11" s="39"/>
+      <c r="A11" s="35"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="35"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="35"/>
+      <c r="I11" s="35"/>
+      <c r="J11" s="35"/>
+      <c r="K11" s="35"/>
+      <c r="L11" s="35"/>
+      <c r="M11" s="35"/>
+      <c r="N11" s="35"/>
+      <c r="O11" s="35"/>
+      <c r="P11" s="35"/>
+      <c r="Q11" s="35"/>
+      <c r="R11" s="35"/>
+      <c r="S11" s="35"/>
+      <c r="T11" s="35"/>
+      <c r="U11" s="35"/>
+      <c r="V11" s="35"/>
+      <c r="W11" s="35"/>
+      <c r="X11" s="35"/>
+      <c r="Y11" s="35"/>
+      <c r="Z11" s="35"/>
+      <c r="AA11" s="35"/>
+      <c r="AB11" s="35"/>
+      <c r="AC11" s="35"/>
+      <c r="AD11" s="35"/>
+      <c r="AE11" s="35"/>
+      <c r="AF11" s="35"/>
+      <c r="AG11" s="35"/>
+      <c r="AH11" s="36"/>
+      <c r="AI11" s="35"/>
+      <c r="AJ11" s="35"/>
+      <c r="AK11" s="34"/>
     </row>
     <row r="12" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A12" s="40"/>
-      <c r="B12" s="40"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="40"/>
-      <c r="J12" s="40"/>
-      <c r="K12" s="40"/>
-      <c r="L12" s="40"/>
-      <c r="M12" s="40"/>
-      <c r="N12" s="40"/>
-      <c r="O12" s="40"/>
-      <c r="P12" s="40"/>
-      <c r="Q12" s="40"/>
-      <c r="R12" s="40"/>
-      <c r="S12" s="40"/>
-      <c r="T12" s="40"/>
-      <c r="U12" s="40"/>
-      <c r="V12" s="40"/>
-      <c r="W12" s="40"/>
-      <c r="X12" s="40"/>
-      <c r="Y12" s="40"/>
-      <c r="Z12" s="40"/>
-      <c r="AA12" s="40"/>
-      <c r="AB12" s="40"/>
-      <c r="AC12" s="40"/>
-      <c r="AD12" s="40"/>
-      <c r="AE12" s="40"/>
-      <c r="AF12" s="40"/>
-      <c r="AG12" s="40"/>
-      <c r="AH12" s="41"/>
-      <c r="AI12" s="40"/>
-      <c r="AJ12" s="40"/>
-      <c r="AK12" s="39"/>
+      <c r="A12" s="35"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
+      <c r="G12" s="35"/>
+      <c r="H12" s="35"/>
+      <c r="I12" s="35"/>
+      <c r="J12" s="35"/>
+      <c r="K12" s="35"/>
+      <c r="L12" s="35"/>
+      <c r="M12" s="35"/>
+      <c r="N12" s="35"/>
+      <c r="O12" s="35"/>
+      <c r="P12" s="35"/>
+      <c r="Q12" s="35"/>
+      <c r="R12" s="35"/>
+      <c r="S12" s="35"/>
+      <c r="T12" s="35"/>
+      <c r="U12" s="35"/>
+      <c r="V12" s="35"/>
+      <c r="W12" s="35"/>
+      <c r="X12" s="35"/>
+      <c r="Y12" s="35"/>
+      <c r="Z12" s="35"/>
+      <c r="AA12" s="35"/>
+      <c r="AB12" s="35"/>
+      <c r="AC12" s="35"/>
+      <c r="AD12" s="35"/>
+      <c r="AE12" s="35"/>
+      <c r="AF12" s="35"/>
+      <c r="AG12" s="35"/>
+      <c r="AH12" s="36"/>
+      <c r="AI12" s="35"/>
+      <c r="AJ12" s="35"/>
+      <c r="AK12" s="34"/>
     </row>
     <row r="13" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A13" s="40"/>
-      <c r="B13" s="40"/>
-      <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="40"/>
-      <c r="G13" s="40"/>
-      <c r="H13" s="40"/>
-      <c r="I13" s="40"/>
-      <c r="J13" s="40"/>
-      <c r="K13" s="40"/>
-      <c r="L13" s="40"/>
-      <c r="M13" s="40"/>
-      <c r="N13" s="40"/>
-      <c r="O13" s="40"/>
-      <c r="P13" s="40"/>
-      <c r="Q13" s="40"/>
-      <c r="R13" s="40"/>
-      <c r="S13" s="40"/>
-      <c r="T13" s="40"/>
-      <c r="U13" s="40"/>
-      <c r="V13" s="40"/>
-      <c r="W13" s="40"/>
-      <c r="X13" s="40"/>
-      <c r="Y13" s="40"/>
-      <c r="Z13" s="40"/>
-      <c r="AA13" s="40"/>
-      <c r="AB13" s="40"/>
-      <c r="AC13" s="40"/>
-      <c r="AD13" s="40"/>
-      <c r="AE13" s="40"/>
-      <c r="AF13" s="40"/>
-      <c r="AG13" s="40"/>
-      <c r="AH13" s="41"/>
-      <c r="AI13" s="40"/>
-      <c r="AJ13" s="40"/>
-      <c r="AK13" s="39"/>
+      <c r="A13" s="35"/>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
+      <c r="G13" s="35"/>
+      <c r="H13" s="35"/>
+      <c r="I13" s="35"/>
+      <c r="J13" s="35"/>
+      <c r="K13" s="35"/>
+      <c r="L13" s="35"/>
+      <c r="M13" s="35"/>
+      <c r="N13" s="35"/>
+      <c r="O13" s="35"/>
+      <c r="P13" s="35"/>
+      <c r="Q13" s="35"/>
+      <c r="R13" s="35"/>
+      <c r="S13" s="35"/>
+      <c r="T13" s="35"/>
+      <c r="U13" s="35"/>
+      <c r="V13" s="35"/>
+      <c r="W13" s="35"/>
+      <c r="X13" s="35"/>
+      <c r="Y13" s="35"/>
+      <c r="Z13" s="35"/>
+      <c r="AA13" s="35"/>
+      <c r="AB13" s="35"/>
+      <c r="AC13" s="35"/>
+      <c r="AD13" s="35"/>
+      <c r="AE13" s="35"/>
+      <c r="AF13" s="35"/>
+      <c r="AG13" s="35"/>
+      <c r="AH13" s="36"/>
+      <c r="AI13" s="35"/>
+      <c r="AJ13" s="35"/>
+      <c r="AK13" s="34"/>
     </row>
     <row r="14" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A14" s="40"/>
-      <c r="B14" s="40"/>
-      <c r="C14" s="40"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="40"/>
-      <c r="G14" s="40"/>
-      <c r="H14" s="40"/>
-      <c r="I14" s="40"/>
-      <c r="J14" s="40"/>
-      <c r="K14" s="40"/>
-      <c r="L14" s="40"/>
-      <c r="M14" s="40"/>
-      <c r="N14" s="40"/>
-      <c r="O14" s="40"/>
-      <c r="P14" s="40"/>
-      <c r="Q14" s="40"/>
-      <c r="R14" s="40"/>
-      <c r="S14" s="40"/>
-      <c r="T14" s="40"/>
-      <c r="U14" s="40"/>
-      <c r="V14" s="40"/>
-      <c r="W14" s="40"/>
-      <c r="X14" s="40"/>
-      <c r="Y14" s="40"/>
-      <c r="Z14" s="40"/>
-      <c r="AA14" s="40"/>
-      <c r="AB14" s="40"/>
-      <c r="AC14" s="40"/>
-      <c r="AD14" s="40"/>
-      <c r="AE14" s="40"/>
-      <c r="AF14" s="40"/>
-      <c r="AG14" s="40"/>
-      <c r="AH14" s="41"/>
-      <c r="AI14" s="40"/>
-      <c r="AJ14" s="40"/>
-      <c r="AK14" s="39"/>
+      <c r="A14" s="35"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
+      <c r="G14" s="35"/>
+      <c r="H14" s="35"/>
+      <c r="I14" s="35"/>
+      <c r="J14" s="35"/>
+      <c r="K14" s="35"/>
+      <c r="L14" s="35"/>
+      <c r="M14" s="35"/>
+      <c r="N14" s="35"/>
+      <c r="O14" s="35"/>
+      <c r="P14" s="35"/>
+      <c r="Q14" s="35"/>
+      <c r="R14" s="35"/>
+      <c r="S14" s="35"/>
+      <c r="T14" s="35"/>
+      <c r="U14" s="35"/>
+      <c r="V14" s="35"/>
+      <c r="W14" s="35"/>
+      <c r="X14" s="35"/>
+      <c r="Y14" s="35"/>
+      <c r="Z14" s="35"/>
+      <c r="AA14" s="35"/>
+      <c r="AB14" s="35"/>
+      <c r="AC14" s="35"/>
+      <c r="AD14" s="35"/>
+      <c r="AE14" s="35"/>
+      <c r="AF14" s="35"/>
+      <c r="AG14" s="35"/>
+      <c r="AH14" s="36"/>
+      <c r="AI14" s="35"/>
+      <c r="AJ14" s="35"/>
+      <c r="AK14" s="34"/>
     </row>
     <row r="15" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A15" s="40"/>
-      <c r="B15" s="40"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="40"/>
-      <c r="J15" s="40"/>
-      <c r="K15" s="40"/>
-      <c r="L15" s="40"/>
-      <c r="M15" s="40"/>
-      <c r="N15" s="40"/>
-      <c r="O15" s="40"/>
-      <c r="P15" s="40"/>
-      <c r="Q15" s="40"/>
-      <c r="R15" s="40"/>
-      <c r="S15" s="40"/>
-      <c r="T15" s="40"/>
-      <c r="U15" s="40"/>
-      <c r="V15" s="40"/>
-      <c r="W15" s="40"/>
-      <c r="X15" s="40"/>
-      <c r="Y15" s="40"/>
-      <c r="Z15" s="40"/>
-      <c r="AA15" s="40"/>
-      <c r="AB15" s="40"/>
-      <c r="AC15" s="40"/>
-      <c r="AD15" s="40"/>
-      <c r="AE15" s="40"/>
-      <c r="AF15" s="40"/>
-      <c r="AG15" s="40"/>
-      <c r="AH15" s="41"/>
-      <c r="AI15" s="40"/>
-      <c r="AJ15" s="40"/>
-      <c r="AK15" s="39"/>
+      <c r="A15" s="35"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35"/>
+      <c r="G15" s="35"/>
+      <c r="H15" s="35"/>
+      <c r="I15" s="35"/>
+      <c r="J15" s="35"/>
+      <c r="K15" s="35"/>
+      <c r="L15" s="35"/>
+      <c r="M15" s="35"/>
+      <c r="N15" s="35"/>
+      <c r="O15" s="35"/>
+      <c r="P15" s="35"/>
+      <c r="Q15" s="35"/>
+      <c r="R15" s="35"/>
+      <c r="S15" s="35"/>
+      <c r="T15" s="35"/>
+      <c r="U15" s="35"/>
+      <c r="V15" s="35"/>
+      <c r="W15" s="35"/>
+      <c r="X15" s="35"/>
+      <c r="Y15" s="35"/>
+      <c r="Z15" s="35"/>
+      <c r="AA15" s="35"/>
+      <c r="AB15" s="35"/>
+      <c r="AC15" s="35"/>
+      <c r="AD15" s="35"/>
+      <c r="AE15" s="35"/>
+      <c r="AF15" s="35"/>
+      <c r="AG15" s="35"/>
+      <c r="AH15" s="36"/>
+      <c r="AI15" s="35"/>
+      <c r="AJ15" s="35"/>
+      <c r="AK15" s="34"/>
     </row>
     <row r="16" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A16" s="40"/>
-      <c r="B16" s="40"/>
-      <c r="C16" s="40"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="40"/>
-      <c r="G16" s="40"/>
-      <c r="H16" s="40"/>
-      <c r="I16" s="40"/>
-      <c r="J16" s="40"/>
-      <c r="K16" s="40"/>
-      <c r="L16" s="40"/>
-      <c r="M16" s="40"/>
-      <c r="N16" s="40"/>
-      <c r="O16" s="40"/>
-      <c r="P16" s="40"/>
-      <c r="Q16" s="40"/>
-      <c r="R16" s="40"/>
-      <c r="S16" s="40"/>
-      <c r="T16" s="40"/>
-      <c r="U16" s="40"/>
-      <c r="V16" s="40"/>
-      <c r="W16" s="40"/>
-      <c r="X16" s="40"/>
-      <c r="Y16" s="40"/>
-      <c r="Z16" s="40"/>
-      <c r="AA16" s="40"/>
-      <c r="AB16" s="40"/>
-      <c r="AC16" s="40"/>
-      <c r="AD16" s="40"/>
-      <c r="AE16" s="40"/>
-      <c r="AF16" s="40"/>
-      <c r="AG16" s="40"/>
-      <c r="AH16" s="41"/>
-      <c r="AI16" s="40"/>
-      <c r="AJ16" s="40"/>
-      <c r="AK16" s="39"/>
+      <c r="A16" s="35"/>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="35"/>
+      <c r="G16" s="35"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="35"/>
+      <c r="J16" s="35"/>
+      <c r="K16" s="35"/>
+      <c r="L16" s="35"/>
+      <c r="M16" s="35"/>
+      <c r="N16" s="35"/>
+      <c r="O16" s="35"/>
+      <c r="P16" s="35"/>
+      <c r="Q16" s="35"/>
+      <c r="R16" s="35"/>
+      <c r="S16" s="35"/>
+      <c r="T16" s="35"/>
+      <c r="U16" s="35"/>
+      <c r="V16" s="35"/>
+      <c r="W16" s="35"/>
+      <c r="X16" s="35"/>
+      <c r="Y16" s="35"/>
+      <c r="Z16" s="35"/>
+      <c r="AA16" s="35"/>
+      <c r="AB16" s="35"/>
+      <c r="AC16" s="35"/>
+      <c r="AD16" s="35"/>
+      <c r="AE16" s="35"/>
+      <c r="AF16" s="35"/>
+      <c r="AG16" s="35"/>
+      <c r="AH16" s="36"/>
+      <c r="AI16" s="35"/>
+      <c r="AJ16" s="35"/>
+      <c r="AK16" s="34"/>
     </row>
     <row r="17" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A17" s="40"/>
-      <c r="B17" s="40"/>
-      <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="40"/>
-      <c r="H17" s="40"/>
-      <c r="I17" s="40"/>
-      <c r="J17" s="40"/>
-      <c r="K17" s="40"/>
-      <c r="L17" s="40"/>
-      <c r="M17" s="40"/>
-      <c r="N17" s="40"/>
-      <c r="O17" s="40"/>
-      <c r="P17" s="40"/>
-      <c r="Q17" s="40"/>
-      <c r="R17" s="40"/>
-      <c r="S17" s="40"/>
-      <c r="T17" s="40"/>
-      <c r="U17" s="40"/>
-      <c r="V17" s="40"/>
-      <c r="W17" s="40"/>
-      <c r="X17" s="40"/>
-      <c r="Y17" s="40"/>
-      <c r="Z17" s="40"/>
-      <c r="AA17" s="40"/>
-      <c r="AB17" s="40"/>
-      <c r="AC17" s="40"/>
-      <c r="AD17" s="40"/>
-      <c r="AE17" s="40"/>
-      <c r="AF17" s="40"/>
-      <c r="AG17" s="40"/>
-      <c r="AH17" s="41"/>
-      <c r="AI17" s="40"/>
-      <c r="AJ17" s="40"/>
-      <c r="AK17" s="39"/>
+      <c r="A17" s="35"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="35"/>
+      <c r="G17" s="35"/>
+      <c r="H17" s="35"/>
+      <c r="I17" s="35"/>
+      <c r="J17" s="35"/>
+      <c r="K17" s="35"/>
+      <c r="L17" s="35"/>
+      <c r="M17" s="35"/>
+      <c r="N17" s="35"/>
+      <c r="O17" s="35"/>
+      <c r="P17" s="35"/>
+      <c r="Q17" s="35"/>
+      <c r="R17" s="35"/>
+      <c r="S17" s="35"/>
+      <c r="T17" s="35"/>
+      <c r="U17" s="35"/>
+      <c r="V17" s="35"/>
+      <c r="W17" s="35"/>
+      <c r="X17" s="35"/>
+      <c r="Y17" s="35"/>
+      <c r="Z17" s="35"/>
+      <c r="AA17" s="35"/>
+      <c r="AB17" s="35"/>
+      <c r="AC17" s="35"/>
+      <c r="AD17" s="35"/>
+      <c r="AE17" s="35"/>
+      <c r="AF17" s="35"/>
+      <c r="AG17" s="35"/>
+      <c r="AH17" s="36"/>
+      <c r="AI17" s="35"/>
+      <c r="AJ17" s="35"/>
+      <c r="AK17" s="34"/>
     </row>
     <row r="18" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A18" s="40"/>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="40"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="40"/>
-      <c r="I18" s="40"/>
-      <c r="J18" s="40"/>
-      <c r="K18" s="40"/>
-      <c r="L18" s="40"/>
-      <c r="M18" s="40"/>
-      <c r="N18" s="40"/>
-      <c r="O18" s="40"/>
-      <c r="P18" s="40"/>
-      <c r="Q18" s="40"/>
-      <c r="R18" s="40"/>
-      <c r="S18" s="40"/>
-      <c r="T18" s="40"/>
-      <c r="U18" s="40"/>
-      <c r="V18" s="40"/>
-      <c r="W18" s="40"/>
-      <c r="X18" s="40"/>
-      <c r="Y18" s="40"/>
-      <c r="Z18" s="40"/>
-      <c r="AA18" s="40"/>
-      <c r="AB18" s="40"/>
-      <c r="AC18" s="40"/>
-      <c r="AD18" s="40"/>
-      <c r="AE18" s="40"/>
-      <c r="AF18" s="40"/>
-      <c r="AG18" s="40"/>
-      <c r="AH18" s="40"/>
-      <c r="AI18" s="40"/>
-      <c r="AJ18" s="40"/>
-      <c r="AK18" s="39"/>
+      <c r="A18" s="35"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="35"/>
+      <c r="G18" s="35"/>
+      <c r="H18" s="35"/>
+      <c r="I18" s="35"/>
+      <c r="J18" s="35"/>
+      <c r="K18" s="35"/>
+      <c r="L18" s="35"/>
+      <c r="M18" s="35"/>
+      <c r="N18" s="35"/>
+      <c r="O18" s="35"/>
+      <c r="P18" s="35"/>
+      <c r="Q18" s="35"/>
+      <c r="R18" s="35"/>
+      <c r="S18" s="35"/>
+      <c r="T18" s="35"/>
+      <c r="U18" s="35"/>
+      <c r="V18" s="35"/>
+      <c r="W18" s="35"/>
+      <c r="X18" s="35"/>
+      <c r="Y18" s="35"/>
+      <c r="Z18" s="35"/>
+      <c r="AA18" s="35"/>
+      <c r="AB18" s="35"/>
+      <c r="AC18" s="35"/>
+      <c r="AD18" s="35"/>
+      <c r="AE18" s="35"/>
+      <c r="AF18" s="35"/>
+      <c r="AG18" s="35"/>
+      <c r="AH18" s="35"/>
+      <c r="AI18" s="35"/>
+      <c r="AJ18" s="35"/>
+      <c r="AK18" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2043,736 +2043,736 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="E1" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="24" t="s">
         <v>47</v>
-      </c>
-      <c r="F1" s="24" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E2" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" s="25" t="s">
         <v>45</v>
-      </c>
-      <c r="F2" s="25" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F3" s="25" t="s">
         <v>147</v>
-      </c>
-      <c r="F3" s="25" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
       <c r="B4" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E4" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="F4" s="25" t="s">
         <v>149</v>
-      </c>
-      <c r="F4" s="25" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E5" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="F5" s="25" t="s">
         <v>151</v>
-      </c>
-      <c r="F5" s="25" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E6" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="F6" s="25" t="s">
         <v>153</v>
-      </c>
-      <c r="F6" s="25" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E7" s="27" t="s">
         <v>8</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
       <c r="B14" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
       <c r="B17" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
       <c r="B18" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
       <c r="B24" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
       <c r="B26" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
       <c r="B27" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
       <c r="B29" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
       <c r="B31" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
       <c r="B32" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5"/>
       <c r="B33" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
       <c r="B36" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5"/>
       <c r="B37" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
       <c r="B40" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5"/>
       <c r="B41" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="12" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="6"/>
       <c r="B45" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="7"/>
       <c r="B46" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="7"/>
       <c r="B48" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
       <c r="B49" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="8"/>
       <c r="B50" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="6"/>
       <c r="B51" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="7"/>
       <c r="B52" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="7"/>
       <c r="B54" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="7"/>
       <c r="B55" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="8"/>
       <c r="B56" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="6"/>
       <c r="B57" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="8"/>
       <c r="B59" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="6"/>
       <c r="B60" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="7"/>
       <c r="B61" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B62" s="7" t="s">
         <v>106</v>
-      </c>
-      <c r="B62" s="7" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="8"/>
       <c r="B63" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="6"/>
       <c r="B64" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
       <c r="B65" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="8"/>
       <c r="B67" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="8"/>
       <c r="B69" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="6"/>
       <c r="B70" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="7"/>
       <c r="B72" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="8"/>
       <c r="B73" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="6"/>
       <c r="B74" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" s="7"/>
       <c r="B76" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="8"/>
       <c r="B77" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B78" s="18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B79" s="19" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B80" s="20" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="9"/>
       <c r="B81" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" s="10"/>
       <c r="B82" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="10"/>
       <c r="B84" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="11"/>
       <c r="B85" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="9"/>
       <c r="B86" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" s="10"/>
       <c r="B88" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="11"/>
       <c r="B89" s="11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="9"/>
       <c r="B90" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="10"/>
       <c r="B92" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="11"/>
       <c r="B93" s="11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="9"/>
       <c r="B94" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" s="10"/>
       <c r="B95" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" s="10"/>
       <c r="B97" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="11"/>
       <c r="B98" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="9"/>
       <c r="B99" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B100" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" s="10"/>
       <c r="B101" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="11"/>
       <c r="B102" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B103" s="21" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="B104" s="21" t="s">
         <v>145</v>
-      </c>
-      <c r="B104" s="21" t="s">
-        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>